<commit_message>
Add Reasoning column to curated workbook
Each row now carries its train of reasoning - calculation arithmetic,
every input figure with its source URL, and caveats - composed at build
time from the deal's research record in outputs/results/, so the
workbook cannot drift from the underlying research.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015Zj6exVHkLABPWezpdGfqF
</commit_message>
<xml_diff>
--- a/precedents/outputs/Deal_Multiples.xlsx
+++ b/precedents/outputs/Deal_Multiples.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Deal Multiples" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Deal Multiples'!$A$1:$F$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Deal Multiples'!$A$1:$G$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -443,7 +443,8 @@
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="62" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="110" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -474,6 +475,11 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Reasoning</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Source</t>
         </is>
       </c>
@@ -500,7 +506,17 @@
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>PUBLISHED EV MULTIPLE: ~31x - Purchase price / CY2023E EBITDA (widely reported alongside the announcement; investor materials also cited a synergy-adjusted multiple) [https://truebluepartners.com/nasdaq-to-acquire-adenza]
+PUBLISHED REVENUE MULTIPLE: ~18x - Purchase price / CY2023E revenue of ~$590M [https://www.cnbc.com/2023/06/12/nasdaq-to-buy-financial-software-firm-adenza-for-10point5-billion.html]
+CALCULATION: $10,500M / $590M 2023E revenue = 17.8x; $590M x 58% adj. EBITDA margin = ~$342M EBITDA; $10,500M / $342M = ~30.7x
+INPUTS: - $10.5B purchase price — Nasdaq press release (8-K exhibit), https://www.sec.gov/Archives/edgar/data/0001120193/000119312523164839/d476077dex991.htm
+- ~$590M 2023E revenue and ~58% adjusted EBITDA margin for Adenza — Nasdaq press release (8-K exhibit), https://www.sec.gov/Archives/edgar/data/0001120193/000119312523164839/d476077dex991.htm
+CAVEATS: Inputs are company-provided 2023 estimates at announcement (revenue growth ~15%, ARR growth ~18% also disclosed); implied math matches the published ~18x revenue / ~31x EBITDA figures</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>CNBC (deal coverage, multiples stated)</t>
         </is>
@@ -528,7 +544,16 @@
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>PUBLISHED EV MULTIPLE: 11x - EV (~GBP 87M) / trailing-twelve-month adjusted EBITDA (~GBP 8M, TTM to July 31, 2023), stated in CoStar's offer press release [https://www.costargroup.com/press-room/2023/costar-group-offers-acquire-leading-uk-residential-property-portal-onthemarket]
+PUBLISHED REVENUE MULTIPLE: 2.5x - EV (~GBP 87M) / trailing-twelve-month revenue (~GBP 35M, TTM to July 31, 2023), stated in CoStar's offer press release [https://www.costargroup.com/press-room/2023/costar-group-offers-acquire-leading-uk-residential-property-portal-onthemarket]
+CALCULATION: GBP 87M EV / GBP 35M TTM revenue = 2.5x; GBP 87M / GBP 8M TTM adjusted EBITDA = 10.9x
+INPUTS: - 110p/share offer, ~GBP 99M equity value, ~GBP 87M EV — https://www.costargroup.com/press-room/2023/costar-group-offers-acquire-leading-uk-residential-property-portal-onthemarket
+- OnTheMarket TTM (to July 31, 2023) revenue ~GBP 35M, adjusted EBITDA ~GBP 8M — same CoStar announcement; OnTheMarket was AIM-listed with audited public accounts</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>CoStar Group offer press release</t>
         </is>
@@ -556,7 +581,16 @@
           <t>~4.9x FY2023E revenue (gross price)</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>PUBLISHED EV MULTIPLE: 13.4x - Net purchase price (~US$190M after tax step-up) / FY2023E normalized EBITDA (~US$14.2M), as stated in Altus Group's press release [https://www.globenewswire.com/news-release/2023/11/09/2777873/0/en/Altus-Group-Enters-into-Agreement-to-Purchase-SitusAMC-s-Commercial-Real-Estate-Valuation-Services-Business.html]
+CALCULATION: US$225.0M / US$46.2M FY2023E revenue = 4.87x; US$190.0M net / US$46.2M = 4.11x. Check on published EBITDA multiple: US$190.0M / US$14.2M = 13.4x (matches)
+INPUTS: - US$225.0M gross / US$190.0M net purchase price — https://www.globenewswire.com/news-release/2023/11/09/2777873/0/en/Altus-Group-Enters-into-Agreement-to-Purchase-SitusAMC-s-Commercial-Real-Estate-Valuation-Services-Business.html
+- REVS FY2023E revenue ~US$46.2M and normalized EBITDA ~US$14.2M — same Altus Group press release
+CAVEATS: Revenue and EBITDA are company-provided fiscal 2023 estimates for the carved-out business, not audited standalone financials.</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Altus Group press release (GlobeNewswire)</t>
         </is>
@@ -580,7 +614,17 @@
       </c>
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>PUBLISHED REVENUE MULTIPLE: 28.8x - Deal value ($1.2B) / SimpleNexus trailing 12-month revenue ($41.6M) [https://www.techbuzznews.com/ncino-acquires-simplenexus-for-1-2-billion/]
+CALCULATION: $1,200M / $41.6M TTM revenue = 28.8x; alternatively $1,200M / ~$54M annualized revenue including October 2021 LBA Ware acquisition = ~22.2x; vs. actual FY2023 SimpleNexus subscription revenue contribution of ~$59.8M ($344.8M total minus $285.0M organic per nCino FY23 results) = ~20.1x
+INPUTS: - Deal value ~$1.2B ($240M cash + ~13.2M NCNO shares) - https://investor.ncino.com/news-releases/news-release-details/ncino-signs-definitive-agreement-acquire-simplenexus/ and https://www.sec.gov/Archives/edgar/data/0001566895/000156689521000036/pressreleaseofncinoinc1116.htm
+- SimpleNexus TTM revenue $41.6M; revenue for year ended Sept 30 2021 of $40.6M; ~$54M annualized incl. LBA Ware - https://www.techbuzznews.com/ncino-acquires-simplenexus-for-1-2-billion/
+- SimpleNexus FY2023 subscription revenue contribution ~$59.8M implied ($344.8M total subscription vs $285.0M organic) - https://investor.ncino.com/news-releases/news-release-details/ncino-reports-fourth-quarter-and-fiscal-year-2023-financial/
+CAVEATS: SimpleNexus was private; its revenue figures come from trade press (TechBuzz News) rather than the nCino press release itself. Stock consideration makes precise deal value time-dependent.</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>TechBuzz News (revenue per trade press; $1.2B price per nCino PR)</t>
         </is>
@@ -604,7 +648,15 @@
           <t>~4.2x P/FY2024 revenue; ~14.1x P/E ($9.4B all-stock)</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>CALCULATION: $9,400M announced equity value / $2,230M Mr. Cooper FY2024 total revenue = 4.2x; $9,400M / $669M FY2024 net income = 14.1x
+INPUTS: - $9.4B all-stock equity value at announcement — https://www.cnbc.com/2025/03/31/mortgage-company-rocket-buying-mr-cooper-in-all-stock-deal-valued-at-9point4-billion.html and https://ir.rocketcompanies.com/news-and-events/press-releases/press-release-details/2025/Mr--Cooper-Americas-Largest-Servicer-Joins-Rocket-the-Nations-Largest-Lender/default.aspx
+- Mr. Cooper FY2024 revenue $2.23B, net income $669.0M — https://finance.yahoo.com/news/mr-cooper-group-full-2024-143804455.html and https://stockanalysis.com/stocks/coop/revenue/ (from 10-K filings)
+CAVEATS: All-stock consideration, so realized value floated (final ~$14.2B at close). EV/Revenue is not the standard lens for an MSR-heavy mortgage servicer; equity-value multiples (P/Revenue, P/E, P/TBV) are more meaningful. Announcement materials published the 35% VWAP premium and exchange ratio but no valuation multiple.</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Rocket Companies press release (financials per COOP filings)</t>
         </is>
@@ -628,7 +680,16 @@
           <t>~4.2x EV/FY2023 segment revenue ($2.45B / ~$579M)</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>CALCULATION: $2,450M / ~$579M FY2023 Digital Banking segment revenue = ~4.2x (~4.4x if the full $100M contingent consideration pays out). EBITDA cross-check: ~38% segment adj. EBITDA margin per management commentary implies ~$220M, giving $2,450M / ~$220M = ~11x.
+INPUTS: - Purchase price $2.45B + up to $100M contingent - Veritas Capital: https://www.veritascapital.com/ncr-voyix-enters-definitive-agreement-to-sell-digital-banking-to-veritas-capital-for-245-billion-purchase-price/ and BusinessWire completion release: https://www.businesswire.com/news/home/20240930825006/en/Veritas-Capital-Completes-Acquisition-of-NCR-Voyixs-Digital-Banking-Business-Rebranding-Business-as-Candescent
+- FY2023 Digital Banking revenue ~$579M and ~1,300 FI clients - press coverage of NCR Voyix's segment disclosures, e.g. https://paymentsindustryintelligence.com/ncr-voyix-sells-to-veritas-for-2-45-billion/ (seller is SEC-reporting; segment detail in NCR Voyix 10-K: https://www.sec.gov/Archives/edgar/data/0000070866/000007086624000014/ncr-20231231.htm)
+- ~38% Digital Banking adj. EBITDA margin - NCR Voyix earnings-call commentary via https://www.investing.com/news/stock-market-news/earnings-call-ncr-voyix-reports-growth-in-software-and-services-for-2023-93CH-3322132
+CAVEATS: SEC.gov and BusinessWire pages were blocked by the network proxy, so the exact 10-K segment figures could not be re-verified on-page; the ~$579M FY2023 revenue is from press coverage of the seller's disclosures (some reports cite $577-579M). EBITDA input is derived from a margin comment, not a stated dollar figure - the ~11x EBITDA multiple is soft. Contingent consideration up to $100M excluded from headline multiple.</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Veritas Capital press release (segment revenue per NCR Voyix disclosures)</t>
         </is>
@@ -652,7 +713,15 @@
           <t>~6.3x EV/FY2024 revenue; ~15.3x EV/FY2024 adj. EBITDA ($2.0B EV)</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>CALCULATION: $2,000M EV / $316.3M FY2024 GAAP revenue = 6.32x; $2,000M EV / $130.7M FY2024 adjusted EBITDA = 15.3x
+INPUTS: - EV ~$2.0B and $20.00/share - MeridianLink press release: https://www.meridianlink.com/press-release/meridianlink-to-be-acquired-by-centerbridge-partners-for-2-0-billion/
+- FY2024 revenue $316.3M and FY2024 adjusted EBITDA $130.7M (41% margin) - MeridianLink Q4/FY2024 earnings release: https://www.businesswire.com/news/home/20250306116917/en/MeridianLink-Reports-Fourth-Quarter-and-Fiscal-Year-2024-Results
+CAVEATS: Multiples computed on FY2024 actuals (last full year pre-announcement). A forward multiple on 2025 guidance would differ; definitive proxy/merger docs would allow a fully diluted EV cross-check.</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>MeridianLink press release (financials per MLNK FY2024 results)</t>
         </is>
@@ -676,7 +745,15 @@
           <t>~15.7x price/CY2021E revenue ($1.1B stock / ~$70M press-reported revenue)</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>CALCULATION: $1,100M all-stock consideration / ~$70M expected CY2021 Technisys revenue = ~15.7x
+INPUTS: - ~$1.1B all-stock deal value (~84M shares at 20-day VWAP) — SoFi press release / 8-K exhibit, https://www.sec.gov/Archives/edgar/data/0001818874/000181887422000014/exhibit991_8-k2222022.htm
+- Technisys expected to deliver approximately $70M of revenue in calendar-year 2021 — announcement-period press coverage, https://www.fool.com/investing/2022/02/25/will-sofis-11b-acquisition-of-technisys-pay-off/
+CAVEATS: The ~$70M CY2021 revenue is a press-reported expectation for a private company, not an audited or company-filed figure; deal value was stock-based and moved with SOFI's share price between announcement and close</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>SoFi 8-K press release (SEC; revenue per announcement-day press)</t>
         </is>
@@ -700,7 +777,16 @@
           <t>~2.2x equity/FY2020 revenue ($468.5M implied 100% / $212.1M)</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>CALCULATION: $422.1M / 0.901 = ~$468.5M implied 100% equity value; $468.5M / $212.1M FY2020 revenue = 2.21x (headline $422.1M / $212.1M = 1.99x; reported $500M EV / $212.1M = 2.36x)
+INPUTS: - Purchase price ~$422.1M in cash for 90.1% of Title365 - Blend Labs S-1 (SEC), https://www.sec.gov/Archives/edgar/data/1855747/000119312521194971/d162671ds1.htm and Meritech S-1 breakdown, https://www.meritechcapital.com/blog/blend-ipo-s-1-breakdown
+- Title365 FY2020 revenue $212.1M - Blend Labs S-1 as summarized by Meritech, https://www.meritechcapital.com/blog/blend-ipo-s-1-breakdown
+- Announcement and structure (90.1% stake, Mr. Cooper retains 9.9%) - PR Newswire, https://www.prnewswire.com/news-releases/blend-to-acquire-title365-from-mr-cooper-group-301247317.html
+CAVEATS: FY2020 was a peak mortgage-refinance year, so the revenue base is cyclical (2019 revenue was far lower); calculation uses equity value as EV proxy on a cash-free/debt-free basis; the ~$500M EV figure appears in press coverage but was not independently re-verified against the 8-K</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Blend Labs S-1 (SEC - both inputs on file)</t>
         </is>
@@ -724,7 +810,15 @@
           <t>~1.0x EV/FY2023 revenue (EUR 330M / ~EUR 340M)</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>CALCULATION: EUR 330M EV / ~EUR 340M FY2023 revenue of the acquired activities = ~0.97x (in USD: ~$357M / ~$368M = ~0.97x)
+INPUTS: - EV EUR 330M - FinTech Futures: https://www.fintechfutures.com/m-a/axway-completes-330m-acquisition-of-sopra-banking-software (citing Axway announcements)
+- Acquired activities revenue ~EUR 340M in FY2023 (~80% of SBS) - The Paypers: https://thepaypers.com/online-mobile-banking/axway-to-acquire-most-sopra-banking-software-activities--1266926 and PAC/SITSI: https://sitsi.pacanalyst.com/sopra-steria-clarifies-its-strategic-direction-by-selling-a-majority-stake-in-sopra-banking-software-sbs/
+CAVEATS: FinTech Futures separately cites EUR 359M standalone revenue for the acquired activities (apparently a 2024 figure at completion), vs ~EUR 340M FY2023 at announcement - implied multiple is ~0.9-1.0x depending on period. No EBITDA disclosed for the perimeter, so no EV/EBITDA. Axway.com and BusinessWire primary releases returned 403 via the network proxy, so exact press-release wording was not independently re-verified; figures are consistent across multiple trade outlets citing those releases.</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>FinTech Futures (completion coverage)</t>
         </is>
@@ -748,7 +842,15 @@
           <t>~8.2x EV/FY2020 revenue (~$240M incl. debt / $29.3M)</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>CALCULATION: $240M transaction value (incl. debt, per acquirer press release) / $29.3M SharpSpring FY2020 total revenue = 8.19x
+INPUTS: - Transaction value ~$240M including outstanding indebtedness - Constant Contact press release, Jun 22, 2021: https://news.constantcontact.com/2021-06-22-Clearlake-Capital-and-Siris-Backed-Constant-Contact-Agrees-to-Acquire-SharpSpring
+- SharpSpring FY2020 total revenue $29.3M (up 29% from $22.7M in 2019) - SharpSpring Q4/FY2020 results: https://investors.sharpspring.com/2021/sharpspring-reports-fourth-quarter-and-full-year-2020-results/
+CAVEATS: Trailing FY2020 revenue basis; the company-stated ~$240M transaction value (including debt) is used as the EV proxy. On a forward basis the multiple would be lower (analyst commentary around announcement cited roughly 7x FY2022E revenue, but that is soft/secondary).</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Constant Contact press release (revenue per SHSP filings)</t>
         </is>
@@ -772,7 +874,15 @@
           <t>~5.6x price/annualized Q3'22 revenue ($225M / ~$40M run-rate)</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>CALCULATION: US$225M / (~US$10M Q3 2022 revenue x 4 = ~US$40M annualized) = ~5.6x
+INPUTS: - US$225M cash purchase price — https://www.prnewswire.com/news-releases/fidelity-national-financial-to-acquire-titlepoint-from-black-knight-301683128.html and FNF 8-K https://www.sec.gov/Archives/edgar/data/0001331875/000133187522000093/ex991pressreleasedatednove.htm
+- TitlePoint ~US$10M revenue in Q3 2022 (incl. $7.2M sensitive to home-buying/origination volumes), per Black Knight, reported by trade press — https://www.inman.com/2022/11/23/fidelity-paying-black-knight-225m-to-bring-titlepoint-back-into-the-fold/ and https://www.housingwire.com/articles/black-knight-to-sell-titlepoint-back-to-fidelity-for-225m/
+CAVEATS: Revenue input is a single quarter (Q3 2022) annualized, not an audited full-year standalone figure; TitlePoint sat inside Black Knight's Data &amp; Analytics segment with no separate annual disclosure. Q3 2022 was also a depressed origination environment, so the run-rate may understate normalized revenue.</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>FNF press release (PR Newswire; revenue per Black Knight disclosure)</t>
         </is>
@@ -796,7 +906,16 @@
           <t>~5.6x price/TTM revenue (~8.9x FY2021; $101M consideration)</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>CALCULATION: US$101M consideration / US$11.4M FY2021 revenue = 8.86x; US$101M / US$18M TTM (to Jul 31, 2022) revenue = 5.6x; US$101M / US$6.7M FY2021 net income = 15.1x
+INPUTS: - Total consideration ~US$101M (US$30M cash + 170M shares) - Voxtur closing press release, https://www.globenewswire.com/news-release/2022/09/22/2520882/0/en/Voxtur-Closes-Acquisition-of-Blue-Water-Financial-Technologies-and-Announces-Expansion-of-Credit-Facilities-and-Private-Placement.html
+- Blue Water FY2021 revenue ~US$11.4M and net income US$6.7M - Voxtur closing press release (same URL) and National Mortgage News, https://www.nationalmortgagenews.com/news/voxtur-to-buy-blue-water-financial-technologies-for-101-million
+- Blue Water TTM (to Jul 31, 2022) revenue ~US$18M, net income ~US$11M - Voxtur closing press release, https://www.globenewswire.com/news-release/2022/09/22/2520882/0/en/Voxtur-Closes-Acquisition-of-Blue-Water-Financial-Technologies-and-Announces-Expansion-of-Credit-Facilities-and-Private-Placement.html
+CAVEATS: Consideration is mostly Voxtur stock, so realized value moved with VXTR share price; financials are acquirer-press-release figures (unaudited); consideration is equity value used as EV proxy - Blue Water net debt not disclosed</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Voxtur closing press release (GlobeNewswire, financials disclosed)</t>
         </is>
@@ -820,7 +939,15 @@
           <t>~5.8x price/2022E revenue ($86.5M / $15M company estimate)</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>CALCULATION: $86.5M closing consideration ($76.5M cash + $10M stock) / $15M company-expected 2022 revenue = 5.77x
+INPUTS: - Closing consideration $76.5M cash + $10M stock - Porch Group press release, Oct 27, 2021: https://www.globenewswire.com/news-release/2021/10/27/2322103/29193/en/Porch-Group-Acquires-Floify-a-Leading-SaaS-Provider-for-Loan-Officers.html (also filed as SEC 8-K Ex-99.1: https://www.sec.gov/Archives/edgar/data/1784535/000110465921130469/tm2130777d1_ex99-1.htm)
+- Floify expected 2022 revenue of $15M (130% net revenue retention as of Q2 2021) - same press release
+CAVEATS: Revenue basis is the company's forward 2022 estimate stated at announcement (Oct 2021), not audited actuals. The stock-guarantee feature and HousingWire's ~$90M headline suggest effective total consideration could be modestly higher than $86.5M. Consideration is purchase price, not a debt-adjusted EV (private target).</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>Porch Group press release (GlobeNewswire)</t>
         </is>
@@ -844,7 +971,15 @@
           <t>~5.4x price/run-rate revenue ($65M / ~$1M per month per CFO)</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>CALCULATION: $65M purchase price / (~$1M per month revenue x 12 = ~$12M annualized run-rate revenue) = ~5.4x
+INPUTS: - $65M all-cash deal value — MeridianLink press release, https://www.businesswire.com/news/home/20221107005914/en/MeridianLink-Announces-Acquisition-of-OpenClose
+- OpenClose revenue of approximately $1M per month, growing at a high-teens rate, per MeridianLink CFO Sean Blitchok on the Q3 2022 earnings call — reported by National Mortgage News, https://www.nationalmortgagenews.com/news/meridianlink-buys-openclose-for-65-million-in-bid-to-reach-more-banks
+CAVEATS: Revenue input is an approximate run-rate stated by acquirer management ('approximately $1 million per month'), not an audited annual figure; annualizing a monthly figure assumes a stable run-rate</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>National Mortgage News (price + CFO revenue commentary)</t>
         </is>
@@ -868,31 +1003,40 @@
           <t>~0.9x price/FY2019 revenue ($40M / $45.1M)</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>CALCULATION: $40M headline consideration / $45.1M FY2019 revenue = 0.89x; on 2020 YTD revenue of &gt;$60M (through ~Oct 2020): $40M / $60M = &lt;0.67x; also ~15.4x FY2019 net income ($40M / $2.6M)
+INPUTS: - Purchase price ~$40M all-cash plus cash-left-in-business adjustment (&gt;=$5M) - Ideanomics definitive agreement press release, https://www.prnewswire.com/news-releases/ideanomics-announces-definitive-agreement-to-acquire-timios-holdings-corp-301171853.html and Seeking Alpha, https://seekingalpha.com/news/3635454-ideanomics-to-acquire-timios-holdings-for-40m
+- Timios FY2019 revenue $45.1M, operating income $4.5M, net income $2.6M - deal disclosures reported via MarketScreener, https://www.marketscreener.com/quote/stock/IDEANOMICS-INC-47133993/news/Ideanomics-Inc-completed-the-acquisition-of-Timios-Inc-from-a-group-of-shareholders-33564470/
+- Timios 2020 YTD revenue over $60M including over $8M in October 2020 - Ideanomics press releases, https://www.prnewswire.com/news-releases/ideanomics-completes-the-acquisition-of-timios-holdings-corp-301205156.html
+CAVEATS: Headline price adjusted upward by cash retained in the business (effective ~$45M, but offset by acquired cash so ~$40M is a reasonable EV proxy); FY2019 revenue predates the deal by a year while the fuller 2020 figure is only a soft 'over $60M YTD'; no full-year 2020 Timios revenue was firmly published at announcement</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>Ideanomics press release (PR Newswire)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F17"/>
+  <autoFilter ref="A1:G17"/>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>